<commit_message>
feat: client feedback round, 35 slides
- Chakira auf der Teamfolie, Callouts und Divider-Zeilen raus
- Zeitstrahl mit neun freigestellten Sparky-Figuren, fette Stichworte, Wendepfeil
- Aktuelles mit drei Szenenbildern, EU-Sternenkreis im Zitatkasten
- Tempo als animierte Wachstumskurve, EU AI Act als Ampel, Ausblick als Treppe
- Prompt-Battle, Praesentationsfolie und Prompt-fuer-morgen entfernt
- Live-Demo neu: zweimal dasselbe Dokument statt Slido-Reparatur
- Wortwolke zum Feedback als vorletzte Folie
- Kahoot: Antwortpositionen gemischt, Bilder neu zugeordnet
</commit_message>
<xml_diff>
--- a/kahoot/kahoot-ki-kompakt.xlsx
+++ b/kahoot/kahoot-ki-kompakt.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +451,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Time limit (sec) – 5, 10, 20, 30, 60, 90, 120, or 240 secs</t>
+          <t>Time limit (sec)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -468,14 +468,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Regel</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Rolle</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Regel</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>Recherche</t>
@@ -490,7 +490,7 @@
         <v>20</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -501,19 +501,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Alles außer S4</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>S1 und S2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>Nur S1, also Öffentliches</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>S1 und S2</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Alles außer S4</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>Alles, wenn man es anonymisiert</t>
@@ -523,7 +523,7 @@
         <v>20</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -567,29 +567,29 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Alle 18 Monate</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Alle 5 Jahre</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Gar nicht mehr</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>Alle 6 Monate</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Alle 18 Monate</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Alle 5 Jahre</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Gar nicht mehr</t>
-        </is>
-      </c>
       <c r="G12" t="n">
         <v>20</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -600,12 +600,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Die Maschine erledigt alles allein</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Die KI arbeitet mit euch, ihr entscheidet</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Die Maschine erledigt alles allein</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -622,7 +622,7 @@
         <v>30</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -633,19 +633,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>1. Januar 2024</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2. Dezember 2027</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>2. August 2026</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>1. Januar 2024</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2. Dezember 2027</t>
-        </is>
-      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>Noch gar nicht</t>
@@ -655,7 +655,7 @@
         <v>20</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -666,29 +666,29 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Ergebnis</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ton</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Auftrag</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>Einschränkung</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Ergebnis</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Ton</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Auftrag</t>
-        </is>
-      </c>
       <c r="G15" t="n">
         <v>20</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -732,19 +732,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Von vorne anfangen</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Das Tool wechseln</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>Per Folgefrage nachbessern</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Von vorne anfangen</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Das Tool wechseln</t>
-        </is>
-      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>Aufgeben</t>
@@ -754,7 +754,7 @@
         <v>20</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -765,14 +765,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Wie einen Taschenrechner</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Wie euren Azubi</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Wie einen Taschenrechner</t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>Wie den Vorstand</t>
@@ -787,7 +787,7 @@
         <v>20</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>